<commit_message>
Concentrate all files in a zip file
</commit_message>
<xml_diff>
--- a/Fiche_Exemple.xlsx
+++ b/Fiche_Exemple.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrateur\Desktop\BOULOT\Fiche de présence\Fiche_de_Paye\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1DF31E3-F53E-4809-BB58-8970D6C3AF37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F45775C-BEB7-4C59-AD6C-6E7BE0583FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{C4044450-EC2F-40B3-BDF9-568C0D9FF30A}"/>
   </bookViews>
@@ -621,20 +621,107 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="46" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -645,131 +732,44 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="46" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1146,897 +1146,897 @@
     <col min="27" max="27" width="2.88671875" customWidth="1"/>
     <col min="28" max="28" width="6.21875" customWidth="1"/>
     <col min="29" max="29" width="2.44140625" customWidth="1"/>
-    <col min="30" max="30" width="6.109375" customWidth="1"/>
+    <col min="30" max="30" width="8.109375" customWidth="1"/>
     <col min="31" max="31" width="7.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:33" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D2" s="62" t="s">
+      <c r="D2" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="41"/>
-      <c r="Q2" s="41"/>
-      <c r="R2" s="41"/>
-      <c r="S2" s="41"/>
-      <c r="T2" s="41"/>
-      <c r="U2" s="41"/>
-      <c r="W2" s="49" t="s">
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
+      <c r="I2" s="51"/>
+      <c r="J2" s="51"/>
+      <c r="K2" s="51"/>
+      <c r="M2" s="37"/>
+      <c r="N2" s="37"/>
+      <c r="O2" s="37"/>
+      <c r="P2" s="37"/>
+      <c r="Q2" s="37"/>
+      <c r="R2" s="37"/>
+      <c r="S2" s="37"/>
+      <c r="T2" s="37"/>
+      <c r="U2" s="37"/>
+      <c r="W2" s="39" t="s">
         <v>22</v>
       </c>
       <c r="X2" s="40"/>
       <c r="Y2" s="40"/>
       <c r="Z2" s="40"/>
-      <c r="AA2" s="50"/>
-      <c r="AB2" s="50"/>
-      <c r="AC2" s="50"/>
-      <c r="AD2" s="50"/>
-      <c r="AE2" s="50"/>
-      <c r="AF2" s="50"/>
-      <c r="AG2" s="51"/>
+      <c r="AA2" s="64"/>
+      <c r="AB2" s="64"/>
+      <c r="AC2" s="64"/>
+      <c r="AD2" s="64"/>
+      <c r="AE2" s="64"/>
+      <c r="AF2" s="64"/>
+      <c r="AG2" s="65"/>
     </row>
     <row r="3" spans="1:33" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="62"/>
-      <c r="M3" s="41"/>
-      <c r="N3" s="41"/>
-      <c r="O3" s="41"/>
-      <c r="P3" s="41"/>
-      <c r="Q3" s="41"/>
-      <c r="R3" s="41"/>
-      <c r="S3" s="41"/>
-      <c r="T3" s="41"/>
-      <c r="U3" s="41"/>
-      <c r="W3" s="47" t="s">
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="51"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="51"/>
+      <c r="K3" s="51"/>
+      <c r="M3" s="37"/>
+      <c r="N3" s="37"/>
+      <c r="O3" s="37"/>
+      <c r="P3" s="37"/>
+      <c r="Q3" s="37"/>
+      <c r="R3" s="37"/>
+      <c r="S3" s="37"/>
+      <c r="T3" s="37"/>
+      <c r="U3" s="37"/>
+      <c r="W3" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="X3" s="85"/>
-      <c r="Y3" s="85"/>
-      <c r="Z3" s="85"/>
-      <c r="AA3" s="85"/>
-      <c r="AB3" s="85"/>
-      <c r="AC3" s="85"/>
-      <c r="AD3" s="85"/>
-      <c r="AE3" s="85"/>
-      <c r="AF3" s="85"/>
-      <c r="AG3" s="48"/>
+      <c r="X3" s="69"/>
+      <c r="Y3" s="69"/>
+      <c r="Z3" s="69"/>
+      <c r="AA3" s="69"/>
+      <c r="AB3" s="69"/>
+      <c r="AC3" s="69"/>
+      <c r="AD3" s="69"/>
+      <c r="AE3" s="69"/>
+      <c r="AF3" s="69"/>
+      <c r="AG3" s="70"/>
     </row>
     <row r="4" spans="1:33" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="62"/>
-      <c r="K4" s="62"/>
-      <c r="M4" s="41"/>
-      <c r="N4" s="41"/>
-      <c r="O4" s="41"/>
-      <c r="P4" s="41"/>
-      <c r="Q4" s="41"/>
-      <c r="R4" s="41"/>
-      <c r="S4" s="41"/>
-      <c r="T4" s="41"/>
-      <c r="U4" s="41"/>
-      <c r="W4" s="45" t="s">
+      <c r="D4" s="51"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="51"/>
+      <c r="G4" s="51"/>
+      <c r="H4" s="51"/>
+      <c r="I4" s="51"/>
+      <c r="J4" s="51"/>
+      <c r="K4" s="51"/>
+      <c r="M4" s="37"/>
+      <c r="N4" s="37"/>
+      <c r="O4" s="37"/>
+      <c r="P4" s="37"/>
+      <c r="Q4" s="37"/>
+      <c r="R4" s="37"/>
+      <c r="S4" s="37"/>
+      <c r="T4" s="37"/>
+      <c r="U4" s="37"/>
+      <c r="W4" s="38" t="s">
         <v>23</v>
       </c>
       <c r="X4" s="35"/>
       <c r="Y4" s="35"/>
       <c r="Z4" s="35"/>
-      <c r="AA4" s="84" t="s">
+      <c r="AA4" s="66" t="s">
         <v>40</v>
       </c>
-      <c r="AB4" s="84"/>
-      <c r="AC4" s="84"/>
-      <c r="AD4" s="84"/>
-      <c r="AE4" s="84"/>
-      <c r="AF4" s="84"/>
-      <c r="AG4" s="46"/>
+      <c r="AB4" s="66"/>
+      <c r="AC4" s="66"/>
+      <c r="AD4" s="66"/>
+      <c r="AE4" s="66"/>
+      <c r="AF4" s="66"/>
+      <c r="AG4" s="67"/>
     </row>
     <row r="5" spans="1:33" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D5" s="62"/>
-      <c r="E5" s="62"/>
-      <c r="F5" s="62"/>
-      <c r="G5" s="62"/>
-      <c r="H5" s="62"/>
-      <c r="I5" s="62"/>
-      <c r="J5" s="62"/>
-      <c r="K5" s="62"/>
-      <c r="M5" s="41"/>
-      <c r="N5" s="41"/>
-      <c r="O5" s="41"/>
-      <c r="P5" s="41"/>
-      <c r="Q5" s="41"/>
-      <c r="R5" s="41"/>
-      <c r="S5" s="41"/>
-      <c r="T5" s="41"/>
-      <c r="U5" s="41"/>
-      <c r="W5" s="47" t="s">
+      <c r="D5" s="51"/>
+      <c r="E5" s="51"/>
+      <c r="F5" s="51"/>
+      <c r="G5" s="51"/>
+      <c r="H5" s="51"/>
+      <c r="I5" s="51"/>
+      <c r="J5" s="51"/>
+      <c r="K5" s="51"/>
+      <c r="M5" s="37"/>
+      <c r="N5" s="37"/>
+      <c r="O5" s="37"/>
+      <c r="P5" s="37"/>
+      <c r="Q5" s="37"/>
+      <c r="R5" s="37"/>
+      <c r="S5" s="37"/>
+      <c r="T5" s="37"/>
+      <c r="U5" s="37"/>
+      <c r="W5" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="X5" s="85"/>
-      <c r="Y5" s="85"/>
-      <c r="Z5" s="85"/>
-      <c r="AA5" s="85"/>
-      <c r="AB5" s="85"/>
-      <c r="AC5" s="85"/>
-      <c r="AD5" s="85"/>
-      <c r="AE5" s="85"/>
-      <c r="AF5" s="85"/>
-      <c r="AG5" s="48"/>
+      <c r="X5" s="69"/>
+      <c r="Y5" s="69"/>
+      <c r="Z5" s="69"/>
+      <c r="AA5" s="69"/>
+      <c r="AB5" s="69"/>
+      <c r="AC5" s="69"/>
+      <c r="AD5" s="69"/>
+      <c r="AE5" s="69"/>
+      <c r="AF5" s="69"/>
+      <c r="AG5" s="70"/>
     </row>
     <row r="6" spans="1:33" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D6" s="62"/>
-      <c r="E6" s="62"/>
-      <c r="F6" s="62"/>
-      <c r="G6" s="62"/>
-      <c r="H6" s="62"/>
-      <c r="I6" s="62"/>
-      <c r="J6" s="62"/>
-      <c r="K6" s="62"/>
-      <c r="M6" s="41"/>
-      <c r="N6" s="41"/>
-      <c r="O6" s="41"/>
-      <c r="P6" s="41"/>
-      <c r="Q6" s="41"/>
-      <c r="R6" s="41"/>
-      <c r="S6" s="41"/>
-      <c r="T6" s="41"/>
-      <c r="U6" s="41"/>
-      <c r="W6" s="45" t="s">
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="51"/>
+      <c r="G6" s="51"/>
+      <c r="H6" s="51"/>
+      <c r="I6" s="51"/>
+      <c r="J6" s="51"/>
+      <c r="K6" s="51"/>
+      <c r="M6" s="37"/>
+      <c r="N6" s="37"/>
+      <c r="O6" s="37"/>
+      <c r="P6" s="37"/>
+      <c r="Q6" s="37"/>
+      <c r="R6" s="37"/>
+      <c r="S6" s="37"/>
+      <c r="T6" s="37"/>
+      <c r="U6" s="37"/>
+      <c r="W6" s="38" t="s">
         <v>19</v>
       </c>
       <c r="X6" s="35"/>
       <c r="Y6" s="35"/>
       <c r="Z6" s="35"/>
-      <c r="AA6" s="84"/>
-      <c r="AB6" s="84"/>
-      <c r="AC6" s="84"/>
-      <c r="AD6" s="84"/>
-      <c r="AE6" s="84"/>
-      <c r="AF6" s="84"/>
-      <c r="AG6" s="46"/>
+      <c r="AA6" s="66"/>
+      <c r="AB6" s="66"/>
+      <c r="AC6" s="66"/>
+      <c r="AD6" s="66"/>
+      <c r="AE6" s="66"/>
+      <c r="AF6" s="66"/>
+      <c r="AG6" s="67"/>
     </row>
     <row r="7" spans="1:33" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D7" s="62"/>
-      <c r="E7" s="62"/>
-      <c r="F7" s="62"/>
-      <c r="G7" s="62"/>
-      <c r="H7" s="62"/>
-      <c r="I7" s="62"/>
-      <c r="J7" s="62"/>
-      <c r="K7" s="62"/>
-      <c r="M7" s="41"/>
-      <c r="N7" s="41"/>
-      <c r="O7" s="41"/>
-      <c r="P7" s="41"/>
-      <c r="Q7" s="41"/>
-      <c r="R7" s="41"/>
-      <c r="S7" s="41"/>
-      <c r="T7" s="41"/>
-      <c r="U7" s="41"/>
-      <c r="W7" s="42" t="s">
+      <c r="D7" s="51"/>
+      <c r="E7" s="51"/>
+      <c r="F7" s="51"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="51"/>
+      <c r="I7" s="51"/>
+      <c r="J7" s="51"/>
+      <c r="K7" s="51"/>
+      <c r="M7" s="37"/>
+      <c r="N7" s="37"/>
+      <c r="O7" s="37"/>
+      <c r="P7" s="37"/>
+      <c r="Q7" s="37"/>
+      <c r="R7" s="37"/>
+      <c r="S7" s="37"/>
+      <c r="T7" s="37"/>
+      <c r="U7" s="37"/>
+      <c r="W7" s="71" t="s">
         <v>18</v>
       </c>
-      <c r="X7" s="43"/>
-      <c r="Y7" s="43"/>
-      <c r="Z7" s="43"/>
-      <c r="AA7" s="43"/>
-      <c r="AB7" s="43"/>
-      <c r="AC7" s="43"/>
-      <c r="AD7" s="43"/>
-      <c r="AE7" s="43"/>
-      <c r="AF7" s="43"/>
-      <c r="AG7" s="44"/>
+      <c r="X7" s="72"/>
+      <c r="Y7" s="72"/>
+      <c r="Z7" s="72"/>
+      <c r="AA7" s="72"/>
+      <c r="AB7" s="72"/>
+      <c r="AC7" s="72"/>
+      <c r="AD7" s="72"/>
+      <c r="AE7" s="72"/>
+      <c r="AF7" s="72"/>
+      <c r="AG7" s="73"/>
     </row>
     <row r="9" spans="1:33" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="65" t="s">
+      <c r="A9" s="75" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="65"/>
-      <c r="C9" s="65"/>
-      <c r="D9" s="65"/>
-      <c r="E9" s="65"/>
-      <c r="F9" s="65"/>
-      <c r="G9" s="65"/>
-      <c r="H9" s="65"/>
-      <c r="I9" s="65"/>
-      <c r="J9" s="65"/>
-      <c r="K9" s="65"/>
-      <c r="L9" s="65"/>
-      <c r="M9" s="65"/>
-      <c r="N9" s="65"/>
-      <c r="O9" s="65"/>
-      <c r="P9" s="65"/>
-      <c r="Q9" s="65"/>
-      <c r="R9" s="65"/>
-      <c r="S9" s="65"/>
-      <c r="T9" s="65"/>
-      <c r="U9" s="65"/>
-      <c r="V9" s="65"/>
-      <c r="W9" s="65"/>
-      <c r="X9" s="65"/>
-      <c r="Y9" s="65"/>
-      <c r="Z9" s="65"/>
-      <c r="AA9" s="65"/>
-      <c r="AB9" s="65"/>
-      <c r="AC9" s="65"/>
-      <c r="AD9" s="65"/>
-      <c r="AE9" s="65"/>
-      <c r="AF9" s="65"/>
-      <c r="AG9" s="65"/>
+      <c r="B9" s="75"/>
+      <c r="C9" s="75"/>
+      <c r="D9" s="75"/>
+      <c r="E9" s="75"/>
+      <c r="F9" s="75"/>
+      <c r="G9" s="75"/>
+      <c r="H9" s="75"/>
+      <c r="I9" s="75"/>
+      <c r="J9" s="75"/>
+      <c r="K9" s="75"/>
+      <c r="L9" s="75"/>
+      <c r="M9" s="75"/>
+      <c r="N9" s="75"/>
+      <c r="O9" s="75"/>
+      <c r="P9" s="75"/>
+      <c r="Q9" s="75"/>
+      <c r="R9" s="75"/>
+      <c r="S9" s="75"/>
+      <c r="T9" s="75"/>
+      <c r="U9" s="75"/>
+      <c r="V9" s="75"/>
+      <c r="W9" s="75"/>
+      <c r="X9" s="75"/>
+      <c r="Y9" s="75"/>
+      <c r="Z9" s="75"/>
+      <c r="AA9" s="75"/>
+      <c r="AB9" s="75"/>
+      <c r="AC9" s="75"/>
+      <c r="AD9" s="75"/>
+      <c r="AE9" s="75"/>
+      <c r="AF9" s="75"/>
+      <c r="AG9" s="75"/>
     </row>
     <row r="10" spans="1:33" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="54">
+      <c r="B10" s="43">
         <v>1</v>
       </c>
-      <c r="C10" s="55"/>
-      <c r="D10" s="55"/>
-      <c r="E10" s="55"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="54">
+      <c r="C10" s="44"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="44"/>
+      <c r="F10" s="45"/>
+      <c r="G10" s="43">
         <v>2</v>
       </c>
-      <c r="H10" s="55"/>
-      <c r="I10" s="55"/>
-      <c r="J10" s="55"/>
-      <c r="K10" s="56"/>
-      <c r="L10" s="54">
+      <c r="H10" s="44"/>
+      <c r="I10" s="44"/>
+      <c r="J10" s="44"/>
+      <c r="K10" s="45"/>
+      <c r="L10" s="43">
         <v>3</v>
       </c>
-      <c r="M10" s="55"/>
-      <c r="N10" s="55"/>
-      <c r="O10" s="55"/>
-      <c r="P10" s="56"/>
-      <c r="Q10" s="54">
+      <c r="M10" s="44"/>
+      <c r="N10" s="44"/>
+      <c r="O10" s="44"/>
+      <c r="P10" s="45"/>
+      <c r="Q10" s="43">
         <v>4</v>
       </c>
-      <c r="R10" s="55"/>
-      <c r="S10" s="55"/>
-      <c r="T10" s="55"/>
-      <c r="U10" s="56"/>
-      <c r="V10" s="54">
+      <c r="R10" s="44"/>
+      <c r="S10" s="44"/>
+      <c r="T10" s="44"/>
+      <c r="U10" s="45"/>
+      <c r="V10" s="43">
         <v>5</v>
       </c>
-      <c r="W10" s="55"/>
-      <c r="X10" s="55"/>
-      <c r="Y10" s="55"/>
-      <c r="Z10" s="56"/>
-      <c r="AA10" s="54">
+      <c r="W10" s="44"/>
+      <c r="X10" s="44"/>
+      <c r="Y10" s="44"/>
+      <c r="Z10" s="45"/>
+      <c r="AA10" s="43">
         <v>6</v>
       </c>
-      <c r="AB10" s="55"/>
-      <c r="AC10" s="55"/>
-      <c r="AD10" s="55"/>
-      <c r="AE10" s="56"/>
-      <c r="AF10" s="81"/>
-      <c r="AG10" s="82"/>
+      <c r="AB10" s="44"/>
+      <c r="AC10" s="44"/>
+      <c r="AD10" s="44"/>
+      <c r="AE10" s="45"/>
+      <c r="AF10" s="59"/>
+      <c r="AG10" s="60"/>
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A11" s="52" t="s">
+      <c r="A11" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="B11" s="63"/>
+      <c r="B11" s="52"/>
       <c r="C11" s="8"/>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
       <c r="F11" s="10"/>
-      <c r="G11" s="57"/>
+      <c r="G11" s="46"/>
       <c r="H11" s="12"/>
       <c r="I11" s="13"/>
       <c r="J11" s="14"/>
       <c r="K11" s="10"/>
-      <c r="L11" s="57"/>
+      <c r="L11" s="46"/>
       <c r="M11" s="18"/>
       <c r="N11" s="19"/>
       <c r="O11" s="20"/>
       <c r="P11" s="10"/>
-      <c r="Q11" s="57"/>
+      <c r="Q11" s="46"/>
       <c r="R11" s="12"/>
       <c r="S11" s="13"/>
       <c r="T11" s="14"/>
       <c r="U11" s="10"/>
-      <c r="V11" s="63"/>
+      <c r="V11" s="52"/>
       <c r="W11" s="12"/>
       <c r="X11" s="13"/>
       <c r="Y11" s="14"/>
       <c r="Z11" s="10"/>
-      <c r="AA11" s="63"/>
+      <c r="AA11" s="52"/>
       <c r="AB11" s="12"/>
       <c r="AC11" s="13"/>
       <c r="AD11" s="14"/>
       <c r="AE11" s="10"/>
-      <c r="AF11" s="76"/>
-      <c r="AG11" s="77"/>
+      <c r="AF11" s="57"/>
+      <c r="AG11" s="58"/>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A12" s="53"/>
-      <c r="B12" s="64"/>
+      <c r="A12" s="42"/>
+      <c r="B12" s="53"/>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
       <c r="F12" s="11"/>
-      <c r="G12" s="58"/>
+      <c r="G12" s="47"/>
       <c r="H12" s="15"/>
       <c r="I12" s="16"/>
       <c r="J12" s="17"/>
       <c r="K12" s="11"/>
-      <c r="L12" s="58"/>
+      <c r="L12" s="47"/>
       <c r="M12" s="21"/>
       <c r="N12" s="22"/>
       <c r="O12" s="23"/>
       <c r="P12" s="11"/>
-      <c r="Q12" s="58"/>
+      <c r="Q12" s="47"/>
       <c r="R12" s="15"/>
       <c r="S12" s="16"/>
       <c r="T12" s="17"/>
       <c r="U12" s="11"/>
-      <c r="V12" s="64"/>
+      <c r="V12" s="53"/>
       <c r="W12" s="15"/>
       <c r="X12" s="16"/>
       <c r="Y12" s="17"/>
       <c r="Z12" s="11"/>
-      <c r="AA12" s="64"/>
+      <c r="AA12" s="53"/>
       <c r="AB12" s="15"/>
       <c r="AC12" s="16"/>
       <c r="AD12" s="17"/>
       <c r="AE12" s="11"/>
-      <c r="AF12" s="76"/>
-      <c r="AG12" s="77"/>
+      <c r="AF12" s="57"/>
+      <c r="AG12" s="58"/>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A13" s="52" t="s">
+      <c r="A13" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="57"/>
+      <c r="B13" s="46"/>
       <c r="C13" s="12"/>
       <c r="D13" s="13"/>
       <c r="E13" s="14"/>
       <c r="F13" s="10"/>
-      <c r="G13" s="57"/>
+      <c r="G13" s="46"/>
       <c r="H13" s="12"/>
       <c r="I13" s="13"/>
       <c r="J13" s="14"/>
       <c r="K13" s="10"/>
-      <c r="L13" s="57"/>
+      <c r="L13" s="46"/>
       <c r="M13" s="12"/>
       <c r="N13" s="13"/>
       <c r="O13" s="14"/>
       <c r="P13" s="10"/>
-      <c r="Q13" s="57"/>
+      <c r="Q13" s="46"/>
       <c r="R13" s="12"/>
       <c r="S13" s="13"/>
       <c r="T13" s="14"/>
       <c r="U13" s="10"/>
-      <c r="V13" s="57"/>
+      <c r="V13" s="46"/>
       <c r="W13" s="12"/>
       <c r="X13" s="13"/>
       <c r="Y13" s="14"/>
       <c r="Z13" s="10"/>
-      <c r="AA13" s="57"/>
+      <c r="AA13" s="46"/>
       <c r="AB13" s="12"/>
       <c r="AC13" s="13"/>
       <c r="AD13" s="14"/>
       <c r="AE13" s="10"/>
-      <c r="AF13" s="78" t="s">
+      <c r="AF13" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="AG13" s="79"/>
+      <c r="AG13" s="62"/>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A14" s="53"/>
-      <c r="B14" s="58"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="47"/>
       <c r="C14" s="15"/>
       <c r="D14" s="16"/>
       <c r="E14" s="17"/>
       <c r="F14" s="11"/>
-      <c r="G14" s="58"/>
+      <c r="G14" s="47"/>
       <c r="H14" s="15"/>
       <c r="I14" s="16"/>
       <c r="J14" s="17"/>
       <c r="K14" s="11"/>
-      <c r="L14" s="58"/>
+      <c r="L14" s="47"/>
       <c r="M14" s="15"/>
       <c r="N14" s="16"/>
       <c r="O14" s="17"/>
       <c r="P14" s="11"/>
-      <c r="Q14" s="58"/>
+      <c r="Q14" s="47"/>
       <c r="R14" s="15"/>
       <c r="S14" s="16"/>
       <c r="T14" s="17"/>
       <c r="U14" s="11"/>
-      <c r="V14" s="58"/>
+      <c r="V14" s="47"/>
       <c r="W14" s="15"/>
       <c r="X14" s="16"/>
       <c r="Y14" s="17"/>
       <c r="Z14" s="11"/>
-      <c r="AA14" s="58"/>
+      <c r="AA14" s="47"/>
       <c r="AB14" s="15"/>
       <c r="AC14" s="16"/>
       <c r="AD14" s="17"/>
       <c r="AE14" s="11"/>
-      <c r="AF14" s="83" t="s">
+      <c r="AF14" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="AG14" s="79"/>
+      <c r="AG14" s="62"/>
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A15" s="52" t="s">
+      <c r="A15" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="57"/>
+      <c r="B15" s="46"/>
       <c r="C15" s="12"/>
       <c r="D15" s="13"/>
       <c r="E15" s="14"/>
       <c r="F15" s="10"/>
-      <c r="G15" s="57"/>
+      <c r="G15" s="46"/>
       <c r="H15" s="12"/>
       <c r="I15" s="13"/>
       <c r="J15" s="14"/>
       <c r="K15" s="10"/>
-      <c r="L15" s="57"/>
+      <c r="L15" s="46"/>
       <c r="M15" s="12"/>
       <c r="N15" s="13"/>
       <c r="O15" s="14"/>
       <c r="P15" s="10"/>
-      <c r="Q15" s="57"/>
+      <c r="Q15" s="46"/>
       <c r="R15" s="12"/>
       <c r="S15" s="13"/>
       <c r="T15" s="14"/>
       <c r="U15" s="10"/>
-      <c r="V15" s="57"/>
+      <c r="V15" s="46"/>
       <c r="W15" s="12"/>
       <c r="X15" s="13"/>
       <c r="Y15" s="14"/>
       <c r="Z15" s="10"/>
-      <c r="AA15" s="57"/>
+      <c r="AA15" s="46"/>
       <c r="AB15" s="12"/>
       <c r="AC15" s="13"/>
       <c r="AD15" s="14"/>
       <c r="AE15" s="10"/>
-      <c r="AF15" s="76"/>
-      <c r="AG15" s="77"/>
+      <c r="AF15" s="57"/>
+      <c r="AG15" s="58"/>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A16" s="53"/>
-      <c r="B16" s="58"/>
+      <c r="A16" s="42"/>
+      <c r="B16" s="47"/>
       <c r="C16" s="15"/>
       <c r="D16" s="16"/>
       <c r="E16" s="17"/>
       <c r="F16" s="11"/>
-      <c r="G16" s="58"/>
+      <c r="G16" s="47"/>
       <c r="H16" s="15"/>
       <c r="I16" s="16"/>
       <c r="J16" s="17"/>
       <c r="K16" s="11"/>
-      <c r="L16" s="58"/>
+      <c r="L16" s="47"/>
       <c r="M16" s="15"/>
       <c r="N16" s="16"/>
       <c r="O16" s="17"/>
       <c r="P16" s="11"/>
-      <c r="Q16" s="58"/>
+      <c r="Q16" s="47"/>
       <c r="R16" s="15"/>
       <c r="S16" s="16"/>
       <c r="T16" s="17"/>
       <c r="U16" s="11"/>
-      <c r="V16" s="58"/>
+      <c r="V16" s="47"/>
       <c r="W16" s="15"/>
       <c r="X16" s="16"/>
       <c r="Y16" s="17"/>
       <c r="Z16" s="11"/>
-      <c r="AA16" s="58"/>
+      <c r="AA16" s="47"/>
       <c r="AB16" s="15"/>
       <c r="AC16" s="16"/>
       <c r="AD16" s="17"/>
       <c r="AE16" s="11"/>
-      <c r="AF16" s="78" t="s">
+      <c r="AF16" s="61" t="s">
         <v>12</v>
       </c>
-      <c r="AG16" s="79"/>
+      <c r="AG16" s="62"/>
     </row>
     <row r="17" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A17" s="52" t="s">
+      <c r="A17" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="57"/>
+      <c r="B17" s="46"/>
       <c r="C17" s="12"/>
       <c r="D17" s="13"/>
       <c r="E17" s="14"/>
       <c r="F17" s="10"/>
-      <c r="G17" s="57"/>
+      <c r="G17" s="46"/>
       <c r="H17" s="12"/>
       <c r="I17" s="13"/>
       <c r="J17" s="14"/>
       <c r="K17" s="10"/>
-      <c r="L17" s="57"/>
+      <c r="L17" s="46"/>
       <c r="M17" s="12"/>
       <c r="N17" s="13"/>
       <c r="O17" s="14"/>
       <c r="P17" s="10"/>
-      <c r="Q17" s="57"/>
+      <c r="Q17" s="46"/>
       <c r="R17" s="12"/>
       <c r="S17" s="13"/>
       <c r="T17" s="14"/>
       <c r="U17" s="10"/>
-      <c r="V17" s="57"/>
+      <c r="V17" s="46"/>
       <c r="W17" s="12"/>
       <c r="X17" s="13"/>
       <c r="Y17" s="14"/>
       <c r="Z17" s="10"/>
-      <c r="AA17" s="57"/>
+      <c r="AA17" s="46"/>
       <c r="AB17" s="12"/>
       <c r="AC17" s="13"/>
       <c r="AD17" s="14"/>
       <c r="AE17" s="10"/>
-      <c r="AF17" s="80" t="s">
+      <c r="AF17" s="86" t="s">
         <v>13</v>
       </c>
-      <c r="AG17" s="79"/>
+      <c r="AG17" s="62"/>
     </row>
     <row r="18" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A18" s="53"/>
-      <c r="B18" s="58"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="47"/>
       <c r="C18" s="15"/>
       <c r="D18" s="16"/>
       <c r="E18" s="17"/>
       <c r="F18" s="11"/>
-      <c r="G18" s="58"/>
+      <c r="G18" s="47"/>
       <c r="H18" s="15"/>
       <c r="I18" s="16"/>
       <c r="J18" s="17"/>
       <c r="K18" s="11"/>
-      <c r="L18" s="58"/>
+      <c r="L18" s="47"/>
       <c r="M18" s="15"/>
       <c r="N18" s="16"/>
       <c r="O18" s="17"/>
       <c r="P18" s="11"/>
-      <c r="Q18" s="58"/>
+      <c r="Q18" s="47"/>
       <c r="R18" s="15"/>
       <c r="S18" s="16"/>
       <c r="T18" s="17"/>
       <c r="U18" s="11"/>
-      <c r="V18" s="58"/>
+      <c r="V18" s="47"/>
       <c r="W18" s="15"/>
       <c r="X18" s="16"/>
       <c r="Y18" s="17"/>
       <c r="Z18" s="11"/>
-      <c r="AA18" s="58"/>
+      <c r="AA18" s="47"/>
       <c r="AB18" s="15"/>
       <c r="AC18" s="16"/>
       <c r="AD18" s="17"/>
       <c r="AE18" s="11"/>
-      <c r="AF18" s="76"/>
-      <c r="AG18" s="77"/>
+      <c r="AF18" s="57"/>
+      <c r="AG18" s="58"/>
     </row>
     <row r="19" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A19" s="52" t="s">
+      <c r="A19" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="B19" s="57"/>
+      <c r="B19" s="46"/>
       <c r="C19" s="12"/>
       <c r="D19" s="13"/>
       <c r="E19" s="14"/>
       <c r="F19" s="10"/>
-      <c r="G19" s="57"/>
+      <c r="G19" s="46"/>
       <c r="H19" s="12"/>
       <c r="I19" s="13"/>
       <c r="J19" s="14"/>
       <c r="K19" s="10"/>
-      <c r="L19" s="57"/>
+      <c r="L19" s="46"/>
       <c r="M19" s="12"/>
       <c r="N19" s="13"/>
       <c r="O19" s="14"/>
       <c r="P19" s="10"/>
-      <c r="Q19" s="57"/>
+      <c r="Q19" s="46"/>
       <c r="R19" s="12"/>
       <c r="S19" s="13"/>
       <c r="T19" s="14"/>
       <c r="U19" s="10"/>
-      <c r="V19" s="63"/>
+      <c r="V19" s="52"/>
       <c r="W19" s="9"/>
       <c r="X19" s="9"/>
       <c r="Y19" s="9"/>
       <c r="Z19" s="10"/>
-      <c r="AA19" s="63"/>
+      <c r="AA19" s="52"/>
       <c r="AB19" s="9"/>
       <c r="AC19" s="9"/>
       <c r="AD19" s="9"/>
       <c r="AE19" s="10"/>
-      <c r="AF19" s="76"/>
-      <c r="AG19" s="77"/>
+      <c r="AF19" s="57"/>
+      <c r="AG19" s="58"/>
     </row>
     <row r="20" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A20" s="53"/>
-      <c r="B20" s="58"/>
+      <c r="A20" s="42"/>
+      <c r="B20" s="47"/>
       <c r="C20" s="15"/>
       <c r="D20" s="16"/>
       <c r="E20" s="17"/>
       <c r="F20" s="11"/>
-      <c r="G20" s="58"/>
+      <c r="G20" s="47"/>
       <c r="H20" s="15"/>
       <c r="I20" s="16"/>
       <c r="J20" s="17"/>
       <c r="K20" s="11"/>
-      <c r="L20" s="58"/>
+      <c r="L20" s="47"/>
       <c r="M20" s="15"/>
       <c r="N20" s="16"/>
       <c r="O20" s="17"/>
       <c r="P20" s="11"/>
-      <c r="Q20" s="58"/>
+      <c r="Q20" s="47"/>
       <c r="R20" s="15"/>
       <c r="S20" s="16"/>
       <c r="T20" s="17"/>
       <c r="U20" s="11"/>
-      <c r="V20" s="64"/>
+      <c r="V20" s="53"/>
       <c r="W20" s="15"/>
       <c r="X20" s="16"/>
       <c r="Y20" s="17"/>
       <c r="Z20" s="11"/>
-      <c r="AA20" s="64"/>
+      <c r="AA20" s="53"/>
       <c r="AB20" s="15"/>
       <c r="AC20" s="16"/>
       <c r="AD20" s="17"/>
       <c r="AE20" s="11"/>
-      <c r="AF20" s="66"/>
-      <c r="AG20" s="67"/>
+      <c r="AF20" s="76"/>
+      <c r="AG20" s="77"/>
     </row>
     <row r="21" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A21" s="52" t="s">
+      <c r="A21" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="B21" s="57"/>
+      <c r="B21" s="46"/>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
       <c r="F21" s="10"/>
-      <c r="G21" s="57"/>
+      <c r="G21" s="46"/>
       <c r="H21" s="9"/>
       <c r="I21" s="9"/>
       <c r="J21" s="9"/>
       <c r="K21" s="10"/>
-      <c r="L21" s="57"/>
+      <c r="L21" s="46"/>
       <c r="M21" s="9"/>
       <c r="N21" s="9"/>
       <c r="O21" s="9"/>
       <c r="P21" s="10"/>
-      <c r="Q21" s="57"/>
+      <c r="Q21" s="46"/>
       <c r="R21" s="9"/>
       <c r="S21" s="9"/>
       <c r="T21" s="9"/>
       <c r="U21" s="10"/>
-      <c r="V21" s="63"/>
+      <c r="V21" s="52"/>
       <c r="W21" s="9"/>
       <c r="X21" s="9"/>
       <c r="Y21" s="9"/>
       <c r="Z21" s="10"/>
-      <c r="AA21" s="63"/>
+      <c r="AA21" s="52"/>
       <c r="AB21" s="9"/>
       <c r="AC21" s="9"/>
       <c r="AD21" s="9"/>
       <c r="AE21" s="10"/>
-      <c r="AF21" s="68" t="s">
+      <c r="AF21" s="78" t="s">
         <v>14</v>
       </c>
-      <c r="AG21" s="69"/>
+      <c r="AG21" s="79"/>
     </row>
     <row r="22" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A22" s="53"/>
-      <c r="B22" s="58"/>
+      <c r="A22" s="42"/>
+      <c r="B22" s="47"/>
       <c r="C22" s="15"/>
       <c r="D22" s="16"/>
       <c r="E22" s="17"/>
       <c r="F22" s="11"/>
-      <c r="G22" s="58"/>
+      <c r="G22" s="47"/>
       <c r="H22" s="15"/>
       <c r="I22" s="16"/>
       <c r="J22" s="17"/>
       <c r="K22" s="11"/>
-      <c r="L22" s="58"/>
+      <c r="L22" s="47"/>
       <c r="M22" s="15"/>
       <c r="N22" s="16"/>
       <c r="O22" s="17"/>
       <c r="P22" s="11"/>
-      <c r="Q22" s="58"/>
+      <c r="Q22" s="47"/>
       <c r="R22" s="15"/>
       <c r="S22" s="16"/>
       <c r="T22" s="17"/>
       <c r="U22" s="11"/>
-      <c r="V22" s="64"/>
+      <c r="V22" s="53"/>
       <c r="W22" s="15"/>
       <c r="X22" s="16"/>
       <c r="Y22" s="17"/>
       <c r="Z22" s="11"/>
-      <c r="AA22" s="64"/>
+      <c r="AA22" s="53"/>
       <c r="AB22" s="15"/>
       <c r="AC22" s="16"/>
       <c r="AD22" s="17"/>
       <c r="AE22" s="11"/>
-      <c r="AF22" s="70"/>
-      <c r="AG22" s="71"/>
+      <c r="AF22" s="80"/>
+      <c r="AG22" s="81"/>
     </row>
     <row r="23" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A23" s="52" t="s">
+      <c r="A23" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="57"/>
+      <c r="B23" s="46"/>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
       <c r="F23" s="10"/>
-      <c r="G23" s="57"/>
+      <c r="G23" s="46"/>
       <c r="H23" s="9"/>
       <c r="I23" s="9"/>
       <c r="J23" s="9"/>
       <c r="K23" s="10"/>
-      <c r="L23" s="57"/>
+      <c r="L23" s="46"/>
       <c r="M23" s="9"/>
       <c r="N23" s="9"/>
       <c r="O23" s="9"/>
       <c r="P23" s="10"/>
-      <c r="Q23" s="57"/>
+      <c r="Q23" s="46"/>
       <c r="R23" s="9"/>
       <c r="S23" s="9"/>
       <c r="T23" s="9"/>
       <c r="U23" s="10"/>
-      <c r="V23" s="63"/>
+      <c r="V23" s="52"/>
       <c r="W23" s="9"/>
       <c r="X23" s="9"/>
       <c r="Y23" s="9"/>
       <c r="Z23" s="10"/>
-      <c r="AA23" s="63"/>
+      <c r="AA23" s="52"/>
       <c r="AB23" s="9"/>
       <c r="AC23" s="9"/>
       <c r="AD23" s="9"/>
       <c r="AE23" s="10"/>
-      <c r="AF23" s="72" t="s">
+      <c r="AF23" s="82" t="s">
         <v>15</v>
       </c>
-      <c r="AG23" s="74" t="s">
+      <c r="AG23" s="84" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="24" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A24" s="53"/>
-      <c r="B24" s="58"/>
+      <c r="A24" s="42"/>
+      <c r="B24" s="47"/>
       <c r="C24" s="15"/>
       <c r="D24" s="16"/>
       <c r="E24" s="17"/>
       <c r="F24" s="11"/>
-      <c r="G24" s="58"/>
+      <c r="G24" s="47"/>
       <c r="H24" s="15"/>
       <c r="I24" s="16"/>
       <c r="J24" s="17"/>
       <c r="K24" s="11"/>
-      <c r="L24" s="58"/>
+      <c r="L24" s="47"/>
       <c r="M24" s="15"/>
       <c r="N24" s="16"/>
       <c r="O24" s="17"/>
       <c r="P24" s="11"/>
-      <c r="Q24" s="58"/>
+      <c r="Q24" s="47"/>
       <c r="R24" s="15"/>
       <c r="S24" s="16"/>
       <c r="T24" s="17"/>
       <c r="U24" s="11"/>
-      <c r="V24" s="64"/>
+      <c r="V24" s="53"/>
       <c r="W24" s="15"/>
       <c r="X24" s="16"/>
       <c r="Y24" s="17"/>
       <c r="Z24" s="11"/>
-      <c r="AA24" s="64"/>
+      <c r="AA24" s="53"/>
       <c r="AB24" s="15"/>
       <c r="AC24" s="16"/>
       <c r="AD24" s="17"/>
       <c r="AE24" s="11"/>
-      <c r="AF24" s="73"/>
-      <c r="AG24" s="75"/>
+      <c r="AF24" s="83"/>
+      <c r="AG24" s="85"/>
     </row>
     <row r="25" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A25" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B25" s="59">
+      <c r="B25" s="48">
         <v>1.1666666666666667</v>
       </c>
-      <c r="C25" s="60"/>
-      <c r="D25" s="60"/>
-      <c r="E25" s="60"/>
-      <c r="F25" s="60"/>
-      <c r="G25" s="59">
+      <c r="C25" s="49"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="48">
         <v>1.4583333333333333</v>
       </c>
-      <c r="H25" s="60"/>
-      <c r="I25" s="60"/>
-      <c r="J25" s="60"/>
-      <c r="K25" s="61"/>
-      <c r="L25" s="59">
+      <c r="H25" s="49"/>
+      <c r="I25" s="49"/>
+      <c r="J25" s="49"/>
+      <c r="K25" s="50"/>
+      <c r="L25" s="48">
         <v>1.1666666666666667</v>
       </c>
-      <c r="M25" s="60"/>
-      <c r="N25" s="60"/>
-      <c r="O25" s="60"/>
-      <c r="P25" s="61"/>
-      <c r="Q25" s="59">
+      <c r="M25" s="49"/>
+      <c r="N25" s="49"/>
+      <c r="O25" s="49"/>
+      <c r="P25" s="50"/>
+      <c r="Q25" s="48">
         <v>1.4583333333333333</v>
       </c>
-      <c r="R25" s="60"/>
-      <c r="S25" s="60"/>
-      <c r="T25" s="60"/>
-      <c r="U25" s="61"/>
-      <c r="V25" s="59">
+      <c r="R25" s="49"/>
+      <c r="S25" s="49"/>
+      <c r="T25" s="49"/>
+      <c r="U25" s="50"/>
+      <c r="V25" s="48">
         <v>1.1666666666666667</v>
       </c>
-      <c r="W25" s="60"/>
-      <c r="X25" s="60"/>
-      <c r="Y25" s="60"/>
-      <c r="Z25" s="61"/>
-      <c r="AA25" s="59">
+      <c r="W25" s="49"/>
+      <c r="X25" s="49"/>
+      <c r="Y25" s="49"/>
+      <c r="Z25" s="50"/>
+      <c r="AA25" s="48">
         <v>1.1666666666666667</v>
       </c>
-      <c r="AB25" s="60"/>
-      <c r="AC25" s="60"/>
-      <c r="AD25" s="60"/>
-      <c r="AE25" s="61"/>
+      <c r="AB25" s="49"/>
+      <c r="AC25" s="49"/>
+      <c r="AD25" s="49"/>
+      <c r="AE25" s="50"/>
       <c r="AF25" s="31">
         <v>6.416666666666667</v>
       </c>
       <c r="AG25" s="32"/>
     </row>
     <row r="26" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="37" t="s">
+      <c r="A26" s="54" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="38"/>
-      <c r="C26" s="38"/>
-      <c r="D26" s="38"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="38"/>
-      <c r="G26" s="38"/>
-      <c r="H26" s="38"/>
-      <c r="I26" s="38"/>
-      <c r="J26" s="38"/>
-      <c r="K26" s="38"/>
-      <c r="L26" s="38"/>
-      <c r="M26" s="38"/>
-      <c r="N26" s="38"/>
-      <c r="O26" s="38"/>
-      <c r="P26" s="38"/>
-      <c r="Q26" s="38"/>
-      <c r="R26" s="38"/>
-      <c r="S26" s="38"/>
-      <c r="T26" s="38"/>
-      <c r="U26" s="38"/>
-      <c r="V26" s="38"/>
-      <c r="W26" s="38"/>
-      <c r="X26" s="38"/>
-      <c r="Y26" s="38"/>
-      <c r="Z26" s="38"/>
-      <c r="AA26" s="38"/>
-      <c r="AB26" s="38"/>
-      <c r="AC26" s="38"/>
-      <c r="AD26" s="38"/>
-      <c r="AE26" s="38"/>
-      <c r="AF26" s="38"/>
-      <c r="AG26" s="39"/>
+      <c r="B26" s="55"/>
+      <c r="C26" s="55"/>
+      <c r="D26" s="55"/>
+      <c r="E26" s="55"/>
+      <c r="F26" s="55"/>
+      <c r="G26" s="55"/>
+      <c r="H26" s="55"/>
+      <c r="I26" s="55"/>
+      <c r="J26" s="55"/>
+      <c r="K26" s="55"/>
+      <c r="L26" s="55"/>
+      <c r="M26" s="55"/>
+      <c r="N26" s="55"/>
+      <c r="O26" s="55"/>
+      <c r="P26" s="55"/>
+      <c r="Q26" s="55"/>
+      <c r="R26" s="55"/>
+      <c r="S26" s="55"/>
+      <c r="T26" s="55"/>
+      <c r="U26" s="55"/>
+      <c r="V26" s="55"/>
+      <c r="W26" s="55"/>
+      <c r="X26" s="55"/>
+      <c r="Y26" s="55"/>
+      <c r="Z26" s="55"/>
+      <c r="AA26" s="55"/>
+      <c r="AB26" s="55"/>
+      <c r="AC26" s="55"/>
+      <c r="AD26" s="55"/>
+      <c r="AE26" s="55"/>
+      <c r="AF26" s="55"/>
+      <c r="AG26" s="56"/>
     </row>
     <row r="27" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A27" s="27" t="s">
@@ -2177,8 +2177,8 @@
         <v>38</v>
       </c>
       <c r="AB30" s="35"/>
-      <c r="AC30" s="86"/>
-      <c r="AD30" s="86"/>
+      <c r="AC30" s="74"/>
+      <c r="AD30" s="74"/>
       <c r="AG30" s="3"/>
     </row>
     <row r="31" spans="1:33" x14ac:dyDescent="0.3">
@@ -2278,8 +2278,8 @@
         <v>39</v>
       </c>
       <c r="AB35" s="35"/>
-      <c r="AC35" s="86"/>
-      <c r="AD35" s="86"/>
+      <c r="AC35" s="74"/>
+      <c r="AD35" s="74"/>
       <c r="AG35" s="3"/>
     </row>
     <row r="36" spans="1:33" x14ac:dyDescent="0.3">
@@ -2367,7 +2367,6 @@
     <mergeCell ref="AF16:AG16"/>
     <mergeCell ref="AF17:AG17"/>
     <mergeCell ref="AF18:AG18"/>
-    <mergeCell ref="AF19:AG19"/>
     <mergeCell ref="AF10:AG10"/>
     <mergeCell ref="AF11:AG11"/>
     <mergeCell ref="AF12:AG12"/>
@@ -2378,19 +2377,6 @@
     <mergeCell ref="AA23:AA24"/>
     <mergeCell ref="AA19:AA20"/>
     <mergeCell ref="AA21:AA22"/>
-    <mergeCell ref="Q30:R30"/>
-    <mergeCell ref="Q35:R35"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="G13:G14"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="L10:P10"/>
-    <mergeCell ref="Q10:U10"/>
     <mergeCell ref="Q25:U25"/>
     <mergeCell ref="B11:B12"/>
     <mergeCell ref="L23:L24"/>
@@ -2399,6 +2385,8 @@
     <mergeCell ref="Q13:Q14"/>
     <mergeCell ref="Q15:Q16"/>
     <mergeCell ref="Q17:Q18"/>
+    <mergeCell ref="A26:AG26"/>
+    <mergeCell ref="AF19:AG19"/>
     <mergeCell ref="D2:K7"/>
     <mergeCell ref="B23:B24"/>
     <mergeCell ref="B25:F25"/>
@@ -2412,20 +2400,17 @@
     <mergeCell ref="Q19:Q20"/>
     <mergeCell ref="Q21:Q22"/>
     <mergeCell ref="Q23:Q24"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="L15:L16"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="L21:L22"/>
-    <mergeCell ref="A26:AG26"/>
-    <mergeCell ref="AA27:AE27"/>
-    <mergeCell ref="AA30:AB30"/>
-    <mergeCell ref="AA35:AB35"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="L10:P10"/>
+    <mergeCell ref="Q10:U10"/>
     <mergeCell ref="M5:U7"/>
     <mergeCell ref="M2:U4"/>
     <mergeCell ref="W6:Z6"/>
@@ -2440,6 +2425,16 @@
     <mergeCell ref="A17:A18"/>
     <mergeCell ref="A19:A20"/>
     <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="L21:L22"/>
     <mergeCell ref="W37:AB37"/>
     <mergeCell ref="M37:P37"/>
     <mergeCell ref="A37:F37"/>
@@ -2454,6 +2449,11 @@
     <mergeCell ref="G30:H30"/>
     <mergeCell ref="G35:H35"/>
     <mergeCell ref="Q27:R27"/>
+    <mergeCell ref="AA35:AB35"/>
+    <mergeCell ref="Q30:R30"/>
+    <mergeCell ref="Q35:R35"/>
+    <mergeCell ref="AA27:AE27"/>
+    <mergeCell ref="AA30:AB30"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.22" right="0" top="0" bottom="0" header="0" footer="0.01"/>

</xml_diff>